<commit_message>
IV consolidation, expected-move scale fix, single DB source
- one BS implementation (bs.py); rnd/breeze_loader become adapters
- expected move: straddle/0.7979 not 0.8*straddle (0.638s -> 1.000s)
- VIX from price_bars INDIAVIX time series, not the 12.0 captures placeholder
- db_config.py is the single source for both stores (SQLite + Postgres)
- retire stale root skew_engine mirror; fix path-dependent test imports
- 4 new test modules; see DECISIONS.md D-SC-01..07
</commit_message>
<xml_diff>
--- a/data_agent/fundamentals/screener_data/JIOFIN.xlsx
+++ b/data_agent/fundamentals/screener_data/JIOFIN.xlsx
@@ -4054,7 +4054,7 @@
         <v>43</v>
       </c>
       <c r="B8">
-        <v>262.70</v>
+        <v>249.05</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -4062,7 +4062,7 @@
         <v>79</v>
       </c>
       <c r="B9">
-        <v>173464.50</v>
+        <v>164838.19</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
@@ -4107,7 +4107,7 @@
         <v>2043.29</v>
       </c>
       <c r="K17">
-        <v>3513.26</v>
+        <v>3520.81</v>
       </c>
     </row>
     <row r="18" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4138,10 +4138,10 @@
         <v>118.94</v>
       </c>
       <c r="J22">
-        <v>221.3</v>
+        <v>223.11</v>
       </c>
       <c r="K22">
-        <v>387.27</v>
+        <v>439.29</v>
       </c>
     </row>
     <row r="23" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4155,7 +4155,10 @@
         <v>161.17</v>
       </c>
       <c r="J23">
-        <v>206.38</v>
+        <v>204.57</v>
+      </c>
+      <c r="K23">
+        <v>647.42</v>
       </c>
     </row>
     <row r="24" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4172,7 +4175,7 @@
         <v>66.98</v>
       </c>
       <c r="K24">
-        <v>821.13</v>
+        <v>121.69</v>
       </c>
     </row>
     <row r="25" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4189,7 +4192,7 @@
         <v>428.45</v>
       </c>
       <c r="K25">
-        <v>381.33</v>
+        <v>373.78</v>
       </c>
     </row>
     <row r="26" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4749,7 +4752,7 @@
         <v>6033.46</v>
       </c>
       <c r="K60">
-        <v>7875.13</v>
+        <v>7845.03</v>
       </c>
     </row>
     <row r="61" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4766,7 +4769,7 @@
         <v>133499.98</v>
       </c>
       <c r="K61">
-        <v>163497.08</v>
+        <v>163466.98</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
@@ -4783,7 +4786,7 @@
         <v>179.92</v>
       </c>
       <c r="K62">
-        <v>418.38</v>
+        <v>326.06</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
@@ -4800,7 +4803,7 @@
         <v>14.47</v>
       </c>
       <c r="K63">
-        <v>12.55</v>
+        <v>104.87</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
@@ -4834,7 +4837,7 @@
         <v>14395.27</v>
       </c>
       <c r="K65">
-        <v>29977.48</v>
+        <v>29947.38</v>
       </c>
     </row>
     <row r="66" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4851,7 +4854,7 @@
         <v>133499.98</v>
       </c>
       <c r="K66">
-        <v>163497.08</v>
+        <v>163466.98</v>
       </c>
     </row>
     <row r="67" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -4904,6 +4907,9 @@
         <v>6353284188.0</v>
       </c>
       <c r="J70">
+        <v>6353141623.0</v>
+      </c>
+      <c r="K70">
         <v>6353141623.0</v>
       </c>
     </row>
@@ -4986,7 +4992,7 @@
         <v>-677.57</v>
       </c>
       <c r="J82">
-        <v>-10083.39</v>
+        <v>-10088.73</v>
       </c>
       <c r="K82">
         <v>-15438.64</v>
@@ -5006,7 +5012,7 @@
         <v>6406.18</v>
       </c>
       <c r="K83">
-        <v>-5696.6</v>
+        <v>-5652.34</v>
       </c>
     </row>
     <row r="84" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -5020,7 +5026,7 @@
         <v>-753.04</v>
       </c>
       <c r="J84">
-        <v>3962.35</v>
+        <v>3967.69</v>
       </c>
       <c r="K84">
         <v>21453.7</v>
@@ -5040,7 +5046,7 @@
         <v>285.14</v>
       </c>
       <c r="K85">
-        <v>318.46</v>
+        <v>362.72</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>